<commit_message>
Crude oil data: spelling, clearer units line, instruction text removed (the page is the instruction)
</commit_message>
<xml_diff>
--- a/docs/files/crude-oil-production.xlsx
+++ b/docs/files/crude-oil-production.xlsx
@@ -400,7 +400,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Parrafin wax</t>
+          <t>Paraffin wax</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -463,21 +463,7 @@
     <row r="10">
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Results above are all given in production quantity in gallons per day (thousands)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>You are a chemical engineer working on a design of a refining process for crude oil stock. You have identified 3 options, which give different outputs. Analyze these outputs to come up with</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>the best process for your company (the one that maximizes profits).</t>
+          <t>Quantities above are production, in thousands of gallons per day</t>
         </is>
       </c>
     </row>

</xml_diff>